<commit_message>
docs(feedback): 4th response — Blingz Kim (5/5 across the board)  New response today from the tester behind GA7Y: auto-contribute, payout-turn notifications, savings-history dashboard requested; clearer error messages suggested. Excel re-exported (4 rows), snapshot + next-phase pipeline updated to reflect the live feedback themes.
</commit_message>
<xml_diff>
--- a/docs/feedback/nova-esusu-feedback-2026-08-19.xlsx
+++ b/docs/feedback/nova-esusu-feedback-2026-08-19.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>Timestamp</t>
   </si>
@@ -88,6 +88,21 @@
   </si>
   <si>
     <t>nope</t>
+  </si>
+  <si>
+    <t>Blingz Kim</t>
+  </si>
+  <si>
+    <t>blingzkim@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GA7YBCGYZT77YMPXBJ65DRY4JXFQ52EAV3B5RZQTCA2HXUTVDG3IQHYW </t>
+  </si>
+  <si>
+    <t>Auto-contribute feature and push notifications when it's my turn to receive the pot. Also a dashboard to track my savings history would be great.</t>
+  </si>
+  <si>
+    <t>The connection was smooth, but I'd like clearer error messages when something fails.</t>
   </si>
 </sst>
 </file>
@@ -234,7 +249,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:J4" displayName="Form_Responses" name="Form_Responses" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:J5" displayName="Form_Responses" name="Form_Responses" id="1">
   <tableColumns count="10">
     <tableColumn name="Timestamp" id="1"/>
     <tableColumn name="Your Name" id="2"/>
@@ -588,6 +603,38 @@
         <v>5.0</v>
       </c>
     </row>
+    <row r="5" ht="22.5" customHeight="1">
+      <c r="A5" s="6">
+        <v>46253.54912510417</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="7">
+        <v>5.0</v>
+      </c>
+      <c r="F5" s="7">
+        <v>5.0</v>
+      </c>
+      <c r="G5" s="7">
+        <v>5.0</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="J5" s="7">
+        <v>5.0</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
docs(feedback): 5th response — Blessing Blingz, 5/5 across the board  The tester who pushed through two fixed-mid-session blockers came back with a perfect form response minutes later. Excel re-exported (5 rows); tester table updated — 5 of 6 external testers have now submitted feedback, all 5/5.
</commit_message>
<xml_diff>
--- a/docs/feedback/nova-esusu-feedback-2026-08-19.xlsx
+++ b/docs/feedback/nova-esusu-feedback-2026-08-19.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t>Timestamp</t>
   </si>
@@ -103,6 +103,21 @@
   </si>
   <si>
     <t>The connection was smooth, but I'd like clearer error messages when something fails.</t>
+  </si>
+  <si>
+    <t>Blessing Blingz</t>
+  </si>
+  <si>
+    <t>blessing19edet@@gmail.com</t>
+  </si>
+  <si>
+    <t>GA2UJ6TEQXIEIQGHXQJSSGI2MIEMBQTMZA3OXZMOKYAGF7WU7TTXKW4S</t>
+  </si>
+  <si>
+    <t>No bugs encountered — everything worked smoothly!</t>
+  </si>
+  <si>
+    <t>Tested basic flow — no issues found so far.</t>
   </si>
 </sst>
 </file>
@@ -249,7 +264,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:J5" displayName="Form_Responses" name="Form_Responses" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:J6" displayName="Form_Responses" name="Form_Responses" id="1">
   <tableColumns count="10">
     <tableColumn name="Timestamp" id="1"/>
     <tableColumn name="Your Name" id="2"/>
@@ -635,6 +650,38 @@
         <v>5.0</v>
       </c>
     </row>
+    <row r="6" ht="22.5" customHeight="1">
+      <c r="A6" s="6">
+        <v>46253.58790097223</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" s="7">
+        <v>5.0</v>
+      </c>
+      <c r="F6" s="7">
+        <v>5.0</v>
+      </c>
+      <c r="G6" s="7">
+        <v>5.0</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="J6" s="7">
+        <v>5.0</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
   <tableParts count="1">

</xml_diff>